<commit_message>
Rev 2.5 Add E5080
</commit_message>
<xml_diff>
--- a/Files/License_descriptions.xlsx
+++ b/Files/License_descriptions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benny\Documents\PycharmProjects\InterlligentTester\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8C045D-716E-4C5B-923A-DE4083A37410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746C2769-A55A-49BF-8E1E-27133E632F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C39CC6A0-95FB-4F21-BB12-2A02E9B9E339}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Name</t>
   </si>
@@ -56,6 +56,42 @@
   </si>
   <si>
     <t>005</t>
+  </si>
+  <si>
+    <t>4M2</t>
+  </si>
+  <si>
+    <t>096</t>
+  </si>
+  <si>
+    <t>080</t>
+  </si>
+  <si>
+    <t>083</t>
+  </si>
+  <si>
+    <t>086</t>
+  </si>
+  <si>
+    <t>090</t>
+  </si>
+  <si>
+    <t>4-port test set, 100 kHz to 32 GHz with second source</t>
+  </si>
+  <si>
+    <t>Spectrum analysis hardware, 100 kHz to 32 GHz</t>
+  </si>
+  <si>
+    <t>Frequency Offset Mode (FOM)</t>
+  </si>
+  <si>
+    <t>Frequency Converter Application (FCA)</t>
+  </si>
+  <si>
+    <t>Gain Compression Application (GCA)</t>
+  </si>
+  <si>
+    <t>Spectrum Analysis Application</t>
   </si>
 </sst>
 </file>
@@ -917,7 +953,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03A9A7D3-F374-463B-99BC-EAE43D03075C}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -979,6 +1015,54 @@
         <v>8</v>
       </c>
     </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>